<commit_message>
Update the 2-problem-and-dataset qmd file
</commit_message>
<xml_diff>
--- a/data/Credit_Update.xlsx
+++ b/data/Credit_Update.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawmt\Documents\R-for-Data-Analyst\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soo\Documents\Rdata\R-for-Data-Analyst\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A271700C-C5EE-4199-8FB2-1412A1E6EFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F135AC-41D6-4869-AAF1-5A44FCD83053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="34605" windowHeight="20985" xr2:uid="{9597F283-FDF1-4DE2-937D-1C7E8A587B22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9597F283-FDF1-4DE2-937D-1C7E8A587B22}"/>
   </bookViews>
   <sheets>
     <sheet name="Credit_Update" sheetId="1" r:id="rId1"/>
@@ -620,6 +620,104 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>229331</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>49909</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>352091</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>130080</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE6AF3D4-A073-2D62-A7DD-7C1F2EB897DB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7115040" y="3832200"/>
+            <a:ext cx="122760" cy="260280"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE6AF3D4-A073-2D62-A7DD-7C1F2EB897DB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7108920" y="3826080"/>
+              <a:ext cx="135000" cy="272520"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-04-29T04:30:38.627"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1 1409,'56'124'0,"0"5"-385,-14-3-639,-8-12 1024,-13 5 0,-18-9 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1810.19">307 601 3265,'0'0'6451,"0"3"-6739,7-3-592,5 0-1729,3 0 0</inkml:trace>
+</inkml:ink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3BEE0E56-4487-4F81-BA55-2D3167CAEF94}" name="Table1" displayName="Table1" ref="A1:L401" totalsRowShown="0">
   <autoFilter ref="A1:L401" xr:uid="{3BEE0E56-4487-4F81-BA55-2D3167CAEF94}"/>
@@ -959,12 +1057,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C8492A8-1F8D-4D08-B6D2-6B273BA34CA6}">
   <dimension ref="A1:L401"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="12" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1002,7 +1111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1040,7 +1149,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1078,7 +1187,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1116,7 +1225,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1154,7 +1263,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1192,7 +1301,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1230,7 +1339,7 @@
         <v>1151</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1268,7 +1377,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1306,7 +1415,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1344,7 +1453,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1382,7 +1491,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1420,7 +1529,7 @@
         <v>1407</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1458,7 +1567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1496,7 +1605,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1534,7 +1643,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1572,7 +1681,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1610,7 +1719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1648,7 +1757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1686,7 +1795,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1724,7 +1833,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1762,7 +1871,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1800,7 +1909,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1838,7 +1947,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1876,7 +1985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1914,7 +2023,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1952,7 +2061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1990,7 +2099,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2028,7 +2137,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2066,7 +2175,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2104,7 +2213,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2142,7 +2251,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2180,7 +2289,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2218,7 +2327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2256,7 +2365,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2294,7 +2403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2332,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2370,7 +2479,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2408,7 +2517,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2446,7 +2555,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2484,7 +2593,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2522,7 +2631,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2560,7 +2669,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2598,7 +2707,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2636,7 +2745,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2674,7 +2783,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2712,7 +2821,7 @@
         <v>1120</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2750,7 +2859,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2788,7 +2897,7 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2826,7 +2935,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2864,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2902,7 +3011,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2940,7 +3049,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2978,7 +3087,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -3016,7 +3125,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3054,7 +3163,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3092,7 +3201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3130,7 +3239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3168,7 +3277,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3206,7 +3315,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3244,7 +3353,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3282,7 +3391,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3320,7 +3429,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3358,7 +3467,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3396,7 +3505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3434,7 +3543,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3472,7 +3581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3510,7 +3619,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3548,7 +3657,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3586,7 +3695,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3624,7 +3733,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3662,7 +3771,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3700,7 +3809,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3738,7 +3847,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3776,7 +3885,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3814,7 +3923,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3852,7 +3961,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3890,7 +3999,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3928,7 +4037,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3966,7 +4075,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -4004,7 +4113,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -4042,7 +4151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -4080,7 +4189,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -4118,7 +4227,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -4156,7 +4265,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -4194,7 +4303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -4232,7 +4341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -4270,7 +4379,7 @@
         <v>1779</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -4308,7 +4417,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -4346,7 +4455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -4384,7 +4493,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -4422,7 +4531,7 @@
         <v>1176</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -4460,7 +4569,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -4498,7 +4607,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -4536,7 +4645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -4574,7 +4683,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -4612,7 +4721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -4650,7 +4759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -4688,7 +4797,7 @@
         <v>1380</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -4726,7 +4835,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -4764,7 +4873,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -4802,7 +4911,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -4840,7 +4949,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -4878,7 +4987,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -4916,7 +5025,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -4954,7 +5063,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -4992,7 +5101,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -5030,7 +5139,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -5068,7 +5177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -5106,7 +5215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -5144,7 +5253,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -5182,7 +5291,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -5220,7 +5329,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -5258,7 +5367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -5296,7 +5405,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -5334,7 +5443,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -5372,7 +5481,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -5410,7 +5519,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -5448,7 +5557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -5486,7 +5595,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -5524,7 +5633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -5562,7 +5671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -5600,7 +5709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -5638,7 +5747,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -5676,7 +5785,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -5714,7 +5823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -5752,7 +5861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -5790,7 +5899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -5828,7 +5937,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -5866,7 +5975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -5904,7 +6013,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -5942,7 +6051,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -5980,7 +6089,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -6018,7 +6127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -6056,7 +6165,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -6094,7 +6203,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -6132,7 +6241,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -6170,7 +6279,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -6208,7 +6317,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -6246,7 +6355,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -6284,7 +6393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -6322,7 +6431,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -6360,7 +6469,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -6398,7 +6507,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -6436,7 +6545,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -6474,7 +6583,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -6512,7 +6621,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -6550,7 +6659,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -6588,7 +6697,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -6626,7 +6735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -6664,7 +6773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -6702,7 +6811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -6740,7 +6849,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -6778,7 +6887,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -6816,7 +6925,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -6854,7 +6963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -6892,7 +7001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -6930,7 +7039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -6968,7 +7077,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -7006,7 +7115,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -7044,7 +7153,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -7082,7 +7191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -7120,7 +7229,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -7158,7 +7267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -7196,7 +7305,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -7234,7 +7343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -7272,7 +7381,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -7310,7 +7419,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -7348,7 +7457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -7386,7 +7495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -7424,7 +7533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -7462,7 +7571,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -7500,7 +7609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -7538,7 +7647,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -7576,7 +7685,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -7614,7 +7723,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -7652,7 +7761,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -7690,7 +7799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -7728,7 +7837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -7766,7 +7875,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -7804,7 +7913,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -7842,7 +7951,7 @@
         <v>1237</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -7880,7 +7989,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -7918,7 +8027,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -7956,7 +8065,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -7994,7 +8103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -8032,7 +8141,7 @@
         <v>1448</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -8070,7 +8179,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -8108,7 +8217,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -8146,7 +8255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -8184,7 +8293,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -8222,7 +8331,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -8260,7 +8369,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -8298,7 +8407,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -8336,7 +8445,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -8374,7 +8483,7 @@
         <v>1426</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -8412,7 +8521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>196</v>
       </c>
@@ -8450,7 +8559,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>197</v>
       </c>
@@ -8488,7 +8597,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>198</v>
       </c>
@@ -8526,7 +8635,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>199</v>
       </c>
@@ -8564,7 +8673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>200</v>
       </c>
@@ -8602,7 +8711,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>201</v>
       </c>
@@ -8640,7 +8749,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>202</v>
       </c>
@@ -8678,7 +8787,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>203</v>
       </c>
@@ -8716,7 +8825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>204</v>
       </c>
@@ -8754,7 +8863,7 @@
         <v>1411</v>
       </c>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>205</v>
       </c>
@@ -8792,7 +8901,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>206</v>
       </c>
@@ -8830,7 +8939,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>207</v>
       </c>
@@ -8868,7 +8977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>208</v>
       </c>
@@ -8906,7 +9015,7 @@
         <v>1216</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>209</v>
       </c>
@@ -8944,7 +9053,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>210</v>
       </c>
@@ -8982,7 +9091,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>211</v>
       </c>
@@ -9020,7 +9129,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>212</v>
       </c>
@@ -9058,7 +9167,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>213</v>
       </c>
@@ -9096,7 +9205,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>214</v>
       </c>
@@ -9134,7 +9243,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>215</v>
       </c>
@@ -9172,7 +9281,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>216</v>
       </c>
@@ -9210,7 +9319,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>217</v>
       </c>
@@ -9248,7 +9357,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>218</v>
       </c>
@@ -9286,7 +9395,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>219</v>
       </c>
@@ -9324,7 +9433,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>220</v>
       </c>
@@ -9362,7 +9471,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>221</v>
       </c>
@@ -9400,7 +9509,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>222</v>
       </c>
@@ -9438,7 +9547,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>223</v>
       </c>
@@ -9476,7 +9585,7 @@
         <v>1549</v>
       </c>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>224</v>
       </c>
@@ -9514,7 +9623,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>225</v>
       </c>
@@ -9552,7 +9661,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>226</v>
       </c>
@@ -9590,7 +9699,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>227</v>
       </c>
@@ -9628,7 +9737,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>228</v>
       </c>
@@ -9666,7 +9775,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>229</v>
       </c>
@@ -9704,7 +9813,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>230</v>
       </c>
@@ -9742,7 +9851,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>231</v>
       </c>
@@ -9780,7 +9889,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>232</v>
       </c>
@@ -9818,7 +9927,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>233</v>
       </c>
@@ -9856,7 +9965,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>234</v>
       </c>
@@ -9894,7 +10003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>235</v>
       </c>
@@ -9932,7 +10041,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>236</v>
       </c>
@@ -9970,7 +10079,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>237</v>
       </c>
@@ -10008,7 +10117,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>238</v>
       </c>
@@ -10046,7 +10155,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>239</v>
       </c>
@@ -10084,7 +10193,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>240</v>
       </c>
@@ -10122,7 +10231,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>241</v>
       </c>
@@ -10160,7 +10269,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>242</v>
       </c>
@@ -10198,7 +10307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>243</v>
       </c>
@@ -10236,7 +10345,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>244</v>
       </c>
@@ -10274,7 +10383,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>245</v>
       </c>
@@ -10312,7 +10421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>246</v>
       </c>
@@ -10350,7 +10459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>247</v>
       </c>
@@ -10388,7 +10497,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>248</v>
       </c>
@@ -10426,7 +10535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>249</v>
       </c>
@@ -10464,7 +10573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>250</v>
       </c>
@@ -10502,7 +10611,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>251</v>
       </c>
@@ -10540,7 +10649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>252</v>
       </c>
@@ -10578,7 +10687,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>253</v>
       </c>
@@ -10616,7 +10725,7 @@
         <v>1355</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>254</v>
       </c>
@@ -10654,7 +10763,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>255</v>
       </c>
@@ -10692,7 +10801,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>256</v>
       </c>
@@ -10730,7 +10839,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>257</v>
       </c>
@@ -10768,7 +10877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>258</v>
       </c>
@@ -10806,7 +10915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>259</v>
       </c>
@@ -10844,7 +10953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>260</v>
       </c>
@@ -10882,7 +10991,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>261</v>
       </c>
@@ -10920,7 +11029,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="263" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>262</v>
       </c>
@@ -10958,7 +11067,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>263</v>
       </c>
@@ -10996,7 +11105,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>264</v>
       </c>
@@ -11034,7 +11143,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>265</v>
       </c>
@@ -11072,7 +11181,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>266</v>
       </c>
@@ -11110,7 +11219,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>267</v>
       </c>
@@ -11148,7 +11257,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>268</v>
       </c>
@@ -11186,7 +11295,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>269</v>
       </c>
@@ -11224,7 +11333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>270</v>
       </c>
@@ -11262,7 +11371,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>271</v>
       </c>
@@ -11300,7 +11409,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>272</v>
       </c>
@@ -11338,7 +11447,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>273</v>
       </c>
@@ -11376,7 +11485,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>274</v>
       </c>
@@ -11414,7 +11523,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>275</v>
       </c>
@@ -11452,7 +11561,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="277" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>276</v>
       </c>
@@ -11490,7 +11599,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>277</v>
       </c>
@@ -11528,7 +11637,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="279" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>278</v>
       </c>
@@ -11566,7 +11675,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>279</v>
       </c>
@@ -11604,7 +11713,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>280</v>
       </c>
@@ -11642,7 +11751,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="282" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>281</v>
       </c>
@@ -11680,7 +11789,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>282</v>
       </c>
@@ -11718,7 +11827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>283</v>
       </c>
@@ -11756,7 +11865,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>284</v>
       </c>
@@ -11794,7 +11903,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>285</v>
       </c>
@@ -11832,7 +11941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>286</v>
       </c>
@@ -11870,7 +11979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>287</v>
       </c>
@@ -11908,7 +12017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>288</v>
       </c>
@@ -11946,7 +12055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>289</v>
       </c>
@@ -11984,7 +12093,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>290</v>
       </c>
@@ -12022,7 +12131,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>291</v>
       </c>
@@ -12060,7 +12169,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>292</v>
       </c>
@@ -12098,7 +12207,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>293</v>
       </c>
@@ -12136,7 +12245,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>294</v>
       </c>
@@ -12174,7 +12283,7 @@
         <v>1677</v>
       </c>
     </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>295</v>
       </c>
@@ -12212,7 +12321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>296</v>
       </c>
@@ -12250,7 +12359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>297</v>
       </c>
@@ -12288,7 +12397,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="299" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>298</v>
       </c>
@@ -12326,7 +12435,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="300" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>299</v>
       </c>
@@ -12364,7 +12473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>300</v>
       </c>
@@ -12402,7 +12511,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="302" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>301</v>
       </c>
@@ -12440,7 +12549,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>302</v>
       </c>
@@ -12478,7 +12587,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="304" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>303</v>
       </c>
@@ -12516,7 +12625,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="305" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>304</v>
       </c>
@@ -12554,7 +12663,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="306" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>305</v>
       </c>
@@ -12592,7 +12701,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="307" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>306</v>
       </c>
@@ -12630,7 +12739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>307</v>
       </c>
@@ -12668,7 +12777,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="309" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>308</v>
       </c>
@@ -12706,7 +12815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>309</v>
       </c>
@@ -12744,7 +12853,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="311" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>310</v>
       </c>
@@ -12782,7 +12891,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="312" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>311</v>
       </c>
@@ -12820,7 +12929,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>312</v>
       </c>
@@ -12858,7 +12967,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="314" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>313</v>
       </c>
@@ -12896,7 +13005,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>314</v>
       </c>
@@ -12934,7 +13043,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="316" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>315</v>
       </c>
@@ -12972,7 +13081,7 @@
         <v>1140</v>
       </c>
     </row>
-    <row r="317" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>316</v>
       </c>
@@ -13010,7 +13119,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="318" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>317</v>
       </c>
@@ -13048,7 +13157,7 @@
         <v>1142</v>
       </c>
     </row>
-    <row r="319" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>318</v>
       </c>
@@ -13086,7 +13195,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="320" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>319</v>
       </c>
@@ -13124,7 +13233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>320</v>
       </c>
@@ -13162,7 +13271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>321</v>
       </c>
@@ -13200,7 +13309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="323" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>322</v>
       </c>
@@ -13238,7 +13347,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="324" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>323</v>
       </c>
@@ -13276,7 +13385,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="325" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>324</v>
       </c>
@@ -13314,7 +13423,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="326" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>325</v>
       </c>
@@ -13352,7 +13461,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="327" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>326</v>
       </c>
@@ -13390,7 +13499,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="328" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>327</v>
       </c>
@@ -13428,7 +13537,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="329" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>328</v>
       </c>
@@ -13466,7 +13575,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="330" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>329</v>
       </c>
@@ -13504,7 +13613,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="331" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>330</v>
       </c>
@@ -13542,7 +13651,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="332" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>331</v>
       </c>
@@ -13580,7 +13689,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="333" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>332</v>
       </c>
@@ -13618,7 +13727,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="334" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>333</v>
       </c>
@@ -13656,7 +13765,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="335" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>334</v>
       </c>
@@ -13694,7 +13803,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="336" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>335</v>
       </c>
@@ -13732,7 +13841,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="337" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>336</v>
       </c>
@@ -13770,7 +13879,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="338" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>337</v>
       </c>
@@ -13808,7 +13917,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="339" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>338</v>
       </c>
@@ -13846,7 +13955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="340" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>339</v>
       </c>
@@ -13884,7 +13993,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="341" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>340</v>
       </c>
@@ -13922,7 +14031,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="342" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>341</v>
       </c>
@@ -13960,7 +14069,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="343" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>342</v>
       </c>
@@ -13998,7 +14107,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="344" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>343</v>
       </c>
@@ -14036,7 +14145,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="345" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>344</v>
       </c>
@@ -14074,7 +14183,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="346" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>345</v>
       </c>
@@ -14112,7 +14221,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="347" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>346</v>
       </c>
@@ -14150,7 +14259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>347</v>
       </c>
@@ -14188,7 +14297,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="349" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>348</v>
       </c>
@@ -14226,7 +14335,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="350" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>349</v>
       </c>
@@ -14264,7 +14373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>350</v>
       </c>
@@ -14302,7 +14411,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="352" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>351</v>
       </c>
@@ -14340,7 +14449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="353" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A353">
         <v>352</v>
       </c>
@@ -14378,7 +14487,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="354" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>353</v>
       </c>
@@ -14416,7 +14525,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="355" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A355">
         <v>354</v>
       </c>
@@ -14454,7 +14563,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="356" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A356">
         <v>355</v>
       </c>
@@ -14492,7 +14601,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="357" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A357">
         <v>356</v>
       </c>
@@ -14530,7 +14639,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="358" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>357</v>
       </c>
@@ -14568,7 +14677,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="359" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A359">
         <v>358</v>
       </c>
@@ -14606,7 +14715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="360" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A360">
         <v>359</v>
       </c>
@@ -14644,7 +14753,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="361" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A361">
         <v>360</v>
       </c>
@@ -14682,7 +14791,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="362" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A362">
         <v>361</v>
       </c>
@@ -14720,7 +14829,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="363" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A363">
         <v>362</v>
       </c>
@@ -14758,7 +14867,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="364" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A364">
         <v>363</v>
       </c>
@@ -14796,7 +14905,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="365" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A365">
         <v>364</v>
       </c>
@@ -14834,7 +14943,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="366" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A366">
         <v>365</v>
       </c>
@@ -14872,7 +14981,7 @@
         <v>1243</v>
       </c>
     </row>
-    <row r="367" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A367">
         <v>366</v>
       </c>
@@ -14910,7 +15019,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="368" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A368">
         <v>367</v>
       </c>
@@ -14948,7 +15057,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="369" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A369">
         <v>368</v>
       </c>
@@ -14986,7 +15095,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="370" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A370">
         <v>369</v>
       </c>
@@ -15024,7 +15133,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="371" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A371">
         <v>370</v>
       </c>
@@ -15062,7 +15171,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="372" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A372">
         <v>371</v>
       </c>
@@ -15100,7 +15209,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="373" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A373">
         <v>372</v>
       </c>
@@ -15138,7 +15247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="374" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A374">
         <v>373</v>
       </c>
@@ -15176,7 +15285,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="375" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A375">
         <v>374</v>
       </c>
@@ -15214,7 +15323,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="376" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A376">
         <v>375</v>
       </c>
@@ -15252,7 +15361,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="377" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A377">
         <v>376</v>
       </c>
@@ -15290,7 +15399,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="378" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A378">
         <v>377</v>
       </c>
@@ -15328,7 +15437,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="379" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>378</v>
       </c>
@@ -15366,7 +15475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="380" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A380">
         <v>379</v>
       </c>
@@ -15404,7 +15513,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="381" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A381">
         <v>380</v>
       </c>
@@ -15442,7 +15551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="382" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A382">
         <v>381</v>
       </c>
@@ -15480,7 +15589,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="383" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A383">
         <v>382</v>
       </c>
@@ -15518,7 +15627,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="384" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A384">
         <v>383</v>
       </c>
@@ -15556,7 +15665,7 @@
         <v>1352</v>
       </c>
     </row>
-    <row r="385" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A385">
         <v>384</v>
       </c>
@@ -15594,7 +15703,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="386" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A386">
         <v>385</v>
       </c>
@@ -15632,7 +15741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="387" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A387">
         <v>386</v>
       </c>
@@ -15670,7 +15779,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="388" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A388">
         <v>387</v>
       </c>
@@ -15708,7 +15817,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="389" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A389">
         <v>388</v>
       </c>
@@ -15746,7 +15855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="390" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A390">
         <v>389</v>
       </c>
@@ -15784,7 +15893,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="391" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A391">
         <v>390</v>
       </c>
@@ -15822,7 +15931,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="392" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A392">
         <v>391</v>
       </c>
@@ -15860,7 +15969,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="393" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A393">
         <v>392</v>
       </c>
@@ -15898,7 +16007,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="394" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A394">
         <v>393</v>
       </c>
@@ -15936,7 +16045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="395" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A395">
         <v>394</v>
       </c>
@@ -15974,7 +16083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="396" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A396">
         <v>395</v>
       </c>
@@ -16012,7 +16121,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="397" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A397">
         <v>396</v>
       </c>
@@ -16050,7 +16159,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="398" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A398">
         <v>397</v>
       </c>
@@ -16088,7 +16197,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="399" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A399">
         <v>398</v>
       </c>
@@ -16126,7 +16235,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="400" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A400">
         <v>399</v>
       </c>
@@ -16164,7 +16273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="401" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>400</v>
       </c>
@@ -16204,8 +16313,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>